<commit_message>
docs: address MVP traceability review feedback
</commit_message>
<xml_diff>
--- a/docs/Traceability_Matrix_Updated.xlsx
+++ b/docs/Traceability_Matrix_Updated.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTM" sheetId="1" r:id="R2e0cb4c9cbac43ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule" sheetId="5" r:id="R0c67ba62d3bd46ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="2" r:id="R5dd4dfbf8d0e4eb9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Links" sheetId="6" r:id="R410dab915d3641ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTM" sheetId="1" r:id="R924fd30ee5fb48d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule" sheetId="5" r:id="R5ce07c4c4e87410c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="2" r:id="R1c2dad797bcf4244"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Links" sheetId="6" r:id="R1d41e94beb44436c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1187,7 +1187,7 @@
         <x:v>BR-12; BR-19; S1; S2; S5; S8</x:v>
       </x:c>
       <x:c r="D13" s="17" t="str">
-        <x:v>MVP; benchmarking recording required; structure pending client clarification</x:v>
+        <x:v>MVP benchmarking support and recording; exact fields, retention behaviour and mandatory-record requirement pending client clarification</x:v>
       </x:c>
       <x:c r="E13" s="17" t="str">
         <x:v>benchmarks table; Benchmark type; repository aggregate read support.</x:v>
@@ -1197,10 +1197,10 @@
         <x:v>HYPERLINK is not implemented. linkLocation=#'Evidence Links'!A1, friendlyName=Issue #45; Issue #46</x:v>
       </x:c>
       <x:c r="G13" s="17" t="str">
-        <x:v>No complete benchmark UI/API save flow or automated benchmark test was found. Client-approved MVP agreement requires benchmarking support; current gap is tracked through Issue #45 and the MVP verification work in Issue #46.</x:v>
+        <x:v>Benchmark-related data structures exist, but no complete entry, save and review workflow or automated benchmark coverage was found. Benchmarking support and recording are part of the approved MVP; the exact fields, retention behaviour and whether a record is mandatory before review or submission remain pending client clarification.</x:v>
       </x:c>
       <x:c r="H13" s="17" t="str">
-        <x:v>Not yet satisfied for the approved MVP; benchmarking data exists but the complete user workflow is not implemented</x:v>
+        <x:v>Partially satisfied; benchmarking support is in the MVP, but the final record structure, retention behaviour and mandatory workflow are not confirmed</x:v>
       </x:c>
     </x:row>
     <x:row r="14" s="4" customFormat="1" ht="28.75" customHeight="1">
@@ -1376,7 +1376,7 @@
         <x:v>BR-19; S1; S2; S5; S8</x:v>
       </x:c>
       <x:c r="D20" s="17" t="str">
-        <x:v>MVP; benchmarking must be recordable; retention structure pending client clarification</x:v>
+        <x:v>MVP benchmarking support and recording; record structure, retention and mandatory-record requirement pending client clarification</x:v>
       </x:c>
       <x:c r="E20" s="17" t="str">
         <x:v>benchmarks table and type exist; repository can read benchmark data in aggregate.</x:v>
@@ -1386,10 +1386,10 @@
         <x:v>HYPERLINK is not implemented. linkLocation=#'Evidence Links'!A1, friendlyName=Issue #45; Issue #46</x:v>
       </x:c>
       <x:c r="G20" s="17" t="str">
-        <x:v>Repository review found no complete benchmark save flow, UI entry point or automated test. Client-approved MVP agreement requires benchmark records with source, differences and notes; current implementation lacks the complete workflow.</x:v>
+        <x:v>Repository review found benchmark-related data structures and aggregate reads, but no complete save flow, user interface or automated test. The exact fields, retention behaviour and whether a benchmark record is mandatory before review or submission remain pending client clarification.</x:v>
       </x:c>
       <x:c r="H20" s="17" t="str">
-        <x:v>Not yet satisfied for the approved MVP; benchmarking recording and retention require implementation</x:v>
+        <x:v>Partially satisfied; benchmark recording is not complete, and the final fields, retention behaviour and mandatory-record requirement remain pending client clarification</x:v>
       </x:c>
     </x:row>
     <x:row r="21" s="4" customFormat="1" ht="28.75" customHeight="1">
@@ -2181,12 +2181,12 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="Ra529d930a0204055"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="R369f5ed760ae4eb1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="Rb9b536702f7c42c4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="Refc4dbfef2904816"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8d04ec782574c08"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cfa4608bf1c41a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2476,10 +2476,10 @@
         <x:v>Benchmark data persistence</x:v>
       </x:c>
       <x:c r="C20" s="23" t="str">
-        <x:v>Confirmed MVP benchmarking recording; retention structure pending client clarification</x:v>
+        <x:v>Confirmed MVP benchmarking support; record structure, retention and mandatory-record requirement pending client clarification</x:v>
       </x:c>
       <x:c r="D20" s="24" t="str">
-        <x:v>The MVP requires benchmark records; the level of structure and retention detail still needs client confirmation. Source: S8.</x:v>
+        <x:v>Benchmarking support and the ability to record benchmark information are part of the approved MVP. The current implementation has benchmark-related data structures and aggregate reads, but no complete save flow, user interface or automated test. The exact fields, retention behaviour and whether a benchmark record is mandatory before review or submission remain pending client clarification. Source: S1, S2, S5, S8.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="20">
@@ -2618,7 +2618,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5bbc27d210944d33"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42ef78be46cc4b2b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2935,7 +2935,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3eedac757df4994"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a5c11ec14594690"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>